<commit_message>
some redunant logging - add motion sensor feature
</commit_message>
<xml_diff>
--- a/Apps/echos_speak_advanced_custom/Attributes and Commands/Working Model comparison tonesto to me v4.xlsx
+++ b/Apps/echos_speak_advanced_custom/Attributes and Commands/Working Model comparison tonesto to me v4.xlsx
@@ -8,17 +8,18 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="G:\GitHub\Hubitat\Apps\echos_speak_advanced_custom\Attributes and Commands\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{568BB4E1-32B1-45DE-B6DC-8563253A75CE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5456E440-60B3-48B8-9D97-2E920E4FA301}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15525" xr2:uid="{F6512DD2-A820-4A52-A892-04532F40851E}"/>
+    <workbookView xWindow="-28920" yWindow="5985" windowWidth="29040" windowHeight="15990" activeTab="1" xr2:uid="{F6512DD2-A820-4A52-A892-04532F40851E}"/>
   </bookViews>
   <sheets>
-    <sheet name="Complete list of Desired" sheetId="6" r:id="rId1"/>
-    <sheet name="Actually Implemented" sheetId="1" r:id="rId2"/>
-    <sheet name="Tonesto7 vds Us" sheetId="2" r:id="rId3"/>
-    <sheet name="Specialty Funtions" sheetId="3" r:id="rId4"/>
-    <sheet name="Tonesto7 content commands" sheetId="4" r:id="rId5"/>
-    <sheet name="Music Commands" sheetId="5" r:id="rId6"/>
+    <sheet name="Complete list of Desired 9-15" sheetId="6" r:id="rId1"/>
+    <sheet name="Completed list 9-16" sheetId="7" r:id="rId2"/>
+    <sheet name="Actually Implemented" sheetId="1" r:id="rId3"/>
+    <sheet name="Tonesto7 vds Us" sheetId="2" r:id="rId4"/>
+    <sheet name="Specialty Funtions" sheetId="3" r:id="rId5"/>
+    <sheet name="Tonesto7 content commands" sheetId="4" r:id="rId6"/>
+    <sheet name="Music Commands" sheetId="5" r:id="rId7"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -44,7 +45,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="427" uniqueCount="178">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="500" uniqueCount="195">
   <si>
     <t>Command</t>
   </si>
@@ -844,13 +845,216 @@
   </si>
   <si>
     <t>as of 9/15/26</t>
+  </si>
+  <si>
+    <t>Capability Comparison &amp; Device Testing Matrix</t>
+  </si>
+  <si>
+    <t>Supported by Echos Speak Server Directly?</t>
+  </si>
+  <si>
+    <t>Hubitat Driver Support Status</t>
+  </si>
+  <si>
+    <t>☑</t>
+  </si>
+  <si>
+    <r>
+      <t>Hard Devices</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve"> (N/A on WHA due to Amazon Restriction)</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t>Hard Devices</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve"> (N/A on WHA)</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t>Hard Devices</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve"> (N/A on WHA due to Amazon Sequence Restriction)</t>
+    </r>
+  </si>
+  <si>
+    <t>Fully</t>
+  </si>
+  <si>
+    <t>☐</t>
+  </si>
+  <si>
+    <r>
+      <t>Hard Devices</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve"> (Untested on WHA)</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t>Hard Devices</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve"> (N/A on WHA stream-dependent)</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t>Failing</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve"> (Failed on Dot &amp; Show, N/A on WHA)</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t>Set Volume (</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Google Sans Text"/>
+        <family val="2"/>
+      </rPr>
+      <t>setVolume</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t>)</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t>Hard Devices</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve"> (N/A on WHA due to Amazon API Restriction)</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t>DND On / Off (</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Google Sans Text"/>
+        <family val="2"/>
+      </rPr>
+      <t>setDNDOn</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t>/</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Google Sans Text"/>
+        <family val="2"/>
+      </rPr>
+      <t>setDNDOff</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t>)</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t>Hard Devices</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve"> (N/A on WHA; targets physical speaker instead)</t>
+    </r>
+  </si>
+  <si>
+    <t>Removed - unncessary</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="7">
+  <fonts count="8">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -898,13 +1102,25 @@
       <name val="Google Sans Text"/>
       <family val="2"/>
     </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF9C0006"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
-  <fills count="2">
+  <fills count="3">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFC7CE"/>
+      </patternFill>
     </fill>
   </fills>
   <borders count="2">
@@ -931,10 +1147,11 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="1">
+  <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="7" fillId="2" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="11">
+  <cellXfs count="16">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -954,9 +1171,6 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
@@ -966,8 +1180,27 @@
     <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
     </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="2" borderId="1" xfId="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
   </cellXfs>
-  <cellStyles count="1">
+  <cellStyles count="2">
+    <cellStyle name="Bad" xfId="1" builtinId="27"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
@@ -1336,7 +1569,7 @@
       <c r="D2" s="5" t="s">
         <v>5</v>
       </c>
-      <c r="E2" s="8" t="s">
+      <c r="E2" s="7" t="s">
         <v>144</v>
       </c>
     </row>
@@ -1367,16 +1600,16 @@
       <c r="D4" s="5" t="s">
         <v>7</v>
       </c>
-      <c r="E4" s="9" t="s">
+      <c r="E4" s="8" t="s">
         <v>113</v>
       </c>
-      <c r="F4" s="9" t="s">
+      <c r="F4" s="8" t="s">
         <v>145</v>
       </c>
-      <c r="G4" s="9" t="s">
+      <c r="G4" s="8" t="s">
         <v>146</v>
       </c>
-      <c r="H4" s="9" t="s">
+      <c r="H4" s="8" t="s">
         <v>147</v>
       </c>
     </row>
@@ -1393,16 +1626,16 @@
       <c r="D5" s="5" t="s">
         <v>118</v>
       </c>
-      <c r="E5" s="9" t="s">
+      <c r="E5" s="8" t="s">
         <v>37</v>
       </c>
-      <c r="F5" s="9" t="s">
+      <c r="F5" s="8" t="s">
         <v>148</v>
       </c>
-      <c r="G5" s="9" t="s">
+      <c r="G5" s="8" t="s">
         <v>148</v>
       </c>
-      <c r="H5" s="9" t="s">
+      <c r="H5" s="8" t="s">
         <v>149</v>
       </c>
     </row>
@@ -1419,16 +1652,16 @@
       <c r="D6" s="5" t="s">
         <v>118</v>
       </c>
-      <c r="E6" s="9" t="s">
+      <c r="E6" s="8" t="s">
         <v>117</v>
       </c>
-      <c r="F6" s="9" t="s">
+      <c r="F6" s="8" t="s">
         <v>150</v>
       </c>
-      <c r="G6" s="9" t="s">
+      <c r="G6" s="8" t="s">
         <v>150</v>
       </c>
-      <c r="H6" s="9" t="s">
+      <c r="H6" s="8" t="s">
         <v>151</v>
       </c>
     </row>
@@ -1445,16 +1678,16 @@
       <c r="D7" s="5" t="s">
         <v>118</v>
       </c>
-      <c r="E7" s="9" t="s">
+      <c r="E7" s="8" t="s">
         <v>42</v>
       </c>
-      <c r="F7" s="9" t="s">
+      <c r="F7" s="8" t="s">
         <v>148</v>
       </c>
-      <c r="G7" s="9" t="s">
+      <c r="G7" s="8" t="s">
         <v>148</v>
       </c>
-      <c r="H7" s="9" t="s">
+      <c r="H7" s="8" t="s">
         <v>152</v>
       </c>
     </row>
@@ -1471,16 +1704,16 @@
       <c r="D8" s="5" t="s">
         <v>118</v>
       </c>
-      <c r="E8" s="9" t="s">
+      <c r="E8" s="8" t="s">
         <v>121</v>
       </c>
-      <c r="F8" s="9" t="s">
+      <c r="F8" s="8" t="s">
         <v>150</v>
       </c>
-      <c r="G8" s="9" t="s">
+      <c r="G8" s="8" t="s">
         <v>150</v>
       </c>
-      <c r="H8" s="9" t="s">
+      <c r="H8" s="8" t="s">
         <v>151</v>
       </c>
     </row>
@@ -1497,16 +1730,16 @@
       <c r="D9" s="5" t="s">
         <v>128</v>
       </c>
-      <c r="E9" s="9" t="s">
+      <c r="E9" s="8" t="s">
         <v>153</v>
       </c>
-      <c r="F9" s="9" t="s">
+      <c r="F9" s="8" t="s">
         <v>148</v>
       </c>
-      <c r="G9" s="9" t="s">
+      <c r="G9" s="8" t="s">
         <v>148</v>
       </c>
-      <c r="H9" s="9" t="s">
+      <c r="H9" s="8" t="s">
         <v>154</v>
       </c>
     </row>
@@ -1523,16 +1756,16 @@
       <c r="D10" s="5" t="s">
         <v>128</v>
       </c>
-      <c r="E10" s="9" t="s">
+      <c r="E10" s="8" t="s">
         <v>155</v>
       </c>
-      <c r="F10" s="9" t="s">
+      <c r="F10" s="8" t="s">
         <v>156</v>
       </c>
-      <c r="G10" s="9" t="s">
+      <c r="G10" s="8" t="s">
         <v>156</v>
       </c>
-      <c r="H10" s="9" t="s">
+      <c r="H10" s="8" t="s">
         <v>151</v>
       </c>
     </row>
@@ -1549,16 +1782,16 @@
       <c r="D11" s="5" t="s">
         <v>128</v>
       </c>
-      <c r="E11" s="9" t="s">
+      <c r="E11" s="8" t="s">
         <v>157</v>
       </c>
-      <c r="F11" s="9" t="s">
+      <c r="F11" s="8" t="s">
         <v>148</v>
       </c>
-      <c r="G11" s="9" t="s">
+      <c r="G11" s="8" t="s">
         <v>148</v>
       </c>
-      <c r="H11" s="10" t="s">
+      <c r="H11" s="9" t="s">
         <v>158</v>
       </c>
     </row>
@@ -1575,16 +1808,16 @@
       <c r="D12" s="5" t="s">
         <v>128</v>
       </c>
-      <c r="E12" s="9" t="s">
+      <c r="E12" s="8" t="s">
         <v>159</v>
       </c>
-      <c r="F12" s="9" t="s">
+      <c r="F12" s="8" t="s">
         <v>148</v>
       </c>
-      <c r="G12" s="9" t="s">
+      <c r="G12" s="8" t="s">
         <v>148</v>
       </c>
-      <c r="H12" s="9" t="s">
+      <c r="H12" s="8" t="s">
         <v>160</v>
       </c>
     </row>
@@ -1601,16 +1834,16 @@
       <c r="D13" s="5" t="s">
         <v>128</v>
       </c>
-      <c r="E13" s="9" t="s">
+      <c r="E13" s="8" t="s">
         <v>161</v>
       </c>
-      <c r="F13" s="9" t="s">
+      <c r="F13" s="8" t="s">
         <v>162</v>
       </c>
-      <c r="G13" s="9" t="s">
+      <c r="G13" s="8" t="s">
         <v>162</v>
       </c>
-      <c r="H13" s="9" t="s">
+      <c r="H13" s="8" t="s">
         <v>163</v>
       </c>
     </row>
@@ -1627,16 +1860,16 @@
       <c r="D14" s="5" t="s">
         <v>118</v>
       </c>
-      <c r="E14" s="9" t="s">
+      <c r="E14" s="8" t="s">
         <v>164</v>
       </c>
-      <c r="F14" s="9" t="s">
+      <c r="F14" s="8" t="s">
         <v>165</v>
       </c>
-      <c r="G14" s="9" t="s">
+      <c r="G14" s="8" t="s">
         <v>165</v>
       </c>
-      <c r="H14" s="10" t="s">
+      <c r="H14" s="9" t="s">
         <v>158</v>
       </c>
     </row>
@@ -1653,16 +1886,16 @@
       <c r="D15" s="5" t="s">
         <v>128</v>
       </c>
-      <c r="E15" s="9" t="s">
+      <c r="E15" s="8" t="s">
         <v>166</v>
       </c>
-      <c r="F15" s="9" t="s">
+      <c r="F15" s="8" t="s">
         <v>148</v>
       </c>
-      <c r="G15" s="9" t="s">
+      <c r="G15" s="8" t="s">
         <v>167</v>
       </c>
-      <c r="H15" s="9" t="s">
+      <c r="H15" s="8" t="s">
         <v>168</v>
       </c>
     </row>
@@ -1679,16 +1912,16 @@
       <c r="D16" s="5" t="s">
         <v>128</v>
       </c>
-      <c r="E16" s="9" t="s">
+      <c r="E16" s="8" t="s">
         <v>169</v>
       </c>
-      <c r="F16" s="9" t="s">
+      <c r="F16" s="8" t="s">
         <v>170</v>
       </c>
-      <c r="G16" s="9" t="s">
+      <c r="G16" s="8" t="s">
         <v>170</v>
       </c>
-      <c r="H16" s="9" t="s">
+      <c r="H16" s="8" t="s">
         <v>168</v>
       </c>
     </row>
@@ -1705,16 +1938,16 @@
       <c r="D17" s="5" t="s">
         <v>128</v>
       </c>
-      <c r="E17" s="9" t="s">
+      <c r="E17" s="8" t="s">
         <v>171</v>
       </c>
-      <c r="F17" s="9" t="s">
+      <c r="F17" s="8" t="s">
         <v>172</v>
       </c>
-      <c r="G17" s="9" t="s">
+      <c r="G17" s="8" t="s">
         <v>172</v>
       </c>
-      <c r="H17" s="9" t="s">
+      <c r="H17" s="8" t="s">
         <v>168</v>
       </c>
     </row>
@@ -1731,16 +1964,16 @@
       <c r="D18" s="5" t="s">
         <v>118</v>
       </c>
-      <c r="E18" s="9" t="s">
+      <c r="E18" s="8" t="s">
         <v>173</v>
       </c>
-      <c r="F18" s="9" t="s">
+      <c r="F18" s="8" t="s">
         <v>148</v>
       </c>
-      <c r="G18" s="9" t="s">
+      <c r="G18" s="8" t="s">
         <v>167</v>
       </c>
-      <c r="H18" s="9" t="s">
+      <c r="H18" s="8" t="s">
         <v>168</v>
       </c>
     </row>
@@ -1757,16 +1990,16 @@
       <c r="D19" s="5" t="s">
         <v>118</v>
       </c>
-      <c r="E19" s="9" t="s">
+      <c r="E19" s="8" t="s">
         <v>174</v>
       </c>
-      <c r="F19" s="9" t="s">
+      <c r="F19" s="8" t="s">
         <v>148</v>
       </c>
-      <c r="G19" s="9" t="s">
+      <c r="G19" s="8" t="s">
         <v>148</v>
       </c>
-      <c r="H19" s="10" t="s">
+      <c r="H19" s="9" t="s">
         <v>158</v>
       </c>
     </row>
@@ -1783,16 +2016,16 @@
       <c r="D20" s="5" t="s">
         <v>25</v>
       </c>
-      <c r="E20" s="9" t="s">
+      <c r="E20" s="8" t="s">
         <v>175</v>
       </c>
-      <c r="F20" s="9" t="s">
+      <c r="F20" s="8" t="s">
         <v>148</v>
       </c>
-      <c r="G20" s="9" t="s">
+      <c r="G20" s="8" t="s">
         <v>148</v>
       </c>
-      <c r="H20" s="9" t="s">
+      <c r="H20" s="8" t="s">
         <v>176</v>
       </c>
     </row>
@@ -1839,10 +2072,10 @@
       </c>
     </row>
     <row r="25" spans="1:8" ht="30" customHeight="1">
-      <c r="A25" s="7" t="s">
+      <c r="A25" s="15" t="s">
         <v>143</v>
       </c>
-      <c r="B25" s="7"/>
+      <c r="B25" s="15"/>
     </row>
     <row r="26" spans="1:8">
       <c r="A26" s="5" t="s">
@@ -1951,6 +2184,283 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{821BB5DA-C0AF-4D58-9389-9D0F22C6E60D}">
+  <dimension ref="A1:D20"/>
+  <sheetFormatPr defaultRowHeight="15"/>
+  <cols>
+    <col min="1" max="1" width="61.7109375" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="14.7109375" style="6" customWidth="1"/>
+    <col min="3" max="3" width="26.28515625" style="6" customWidth="1"/>
+    <col min="4" max="4" width="65.28515625" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:4" ht="17.25">
+      <c r="A1" s="7" t="s">
+        <v>178</v>
+      </c>
+    </row>
+    <row r="2" spans="1:4" ht="15.75" thickBot="1">
+      <c r="A2" s="10"/>
+    </row>
+    <row r="3" spans="1:4" ht="48" customHeight="1" thickBot="1">
+      <c r="A3" s="8" t="s">
+        <v>113</v>
+      </c>
+      <c r="B3" s="12" t="s">
+        <v>114</v>
+      </c>
+      <c r="C3" s="12" t="s">
+        <v>179</v>
+      </c>
+      <c r="D3" s="11" t="s">
+        <v>180</v>
+      </c>
+    </row>
+    <row r="4" spans="1:4" ht="15.75" thickBot="1">
+      <c r="A4" s="8" t="s">
+        <v>37</v>
+      </c>
+      <c r="B4" s="13" t="s">
+        <v>181</v>
+      </c>
+      <c r="C4" s="13" t="s">
+        <v>181</v>
+      </c>
+      <c r="D4" s="11" t="s">
+        <v>182</v>
+      </c>
+    </row>
+    <row r="5" spans="1:4" ht="15.75" thickBot="1">
+      <c r="A5" s="8" t="s">
+        <v>117</v>
+      </c>
+      <c r="B5" s="13" t="s">
+        <v>181</v>
+      </c>
+      <c r="C5" s="13" t="s">
+        <v>181</v>
+      </c>
+      <c r="D5" s="11" t="s">
+        <v>183</v>
+      </c>
+    </row>
+    <row r="6" spans="1:4" ht="15.75" thickBot="1">
+      <c r="A6" s="8" t="s">
+        <v>42</v>
+      </c>
+      <c r="B6" s="13" t="s">
+        <v>181</v>
+      </c>
+      <c r="C6" s="13" t="s">
+        <v>181</v>
+      </c>
+      <c r="D6" s="11" t="s">
+        <v>184</v>
+      </c>
+    </row>
+    <row r="7" spans="1:4" ht="15.75" thickBot="1">
+      <c r="A7" s="8" t="s">
+        <v>121</v>
+      </c>
+      <c r="B7" s="13" t="s">
+        <v>181</v>
+      </c>
+      <c r="C7" s="13" t="s">
+        <v>181</v>
+      </c>
+      <c r="D7" s="11" t="s">
+        <v>183</v>
+      </c>
+    </row>
+    <row r="8" spans="1:4" ht="15.75" thickBot="1">
+      <c r="A8" s="8" t="s">
+        <v>153</v>
+      </c>
+      <c r="B8" s="13" t="s">
+        <v>181</v>
+      </c>
+      <c r="C8" s="13" t="s">
+        <v>181</v>
+      </c>
+      <c r="D8" s="11" t="s">
+        <v>194</v>
+      </c>
+    </row>
+    <row r="9" spans="1:4" ht="15.75" thickBot="1">
+      <c r="A9" s="8" t="s">
+        <v>155</v>
+      </c>
+      <c r="B9" s="13" t="s">
+        <v>181</v>
+      </c>
+      <c r="C9" s="13" t="s">
+        <v>181</v>
+      </c>
+      <c r="D9" s="11" t="s">
+        <v>183</v>
+      </c>
+    </row>
+    <row r="10" spans="1:4" ht="15.75" thickBot="1">
+      <c r="A10" s="8" t="s">
+        <v>157</v>
+      </c>
+      <c r="B10" s="13" t="s">
+        <v>181</v>
+      </c>
+      <c r="C10" s="13" t="s">
+        <v>181</v>
+      </c>
+      <c r="D10" s="11" t="s">
+        <v>187</v>
+      </c>
+    </row>
+    <row r="11" spans="1:4" ht="15.75" thickBot="1">
+      <c r="A11" s="8" t="s">
+        <v>159</v>
+      </c>
+      <c r="B11" s="13" t="s">
+        <v>181</v>
+      </c>
+      <c r="C11" s="13" t="s">
+        <v>181</v>
+      </c>
+      <c r="D11" s="11" t="s">
+        <v>185</v>
+      </c>
+    </row>
+    <row r="12" spans="1:4" ht="15.75" thickBot="1">
+      <c r="A12" s="8" t="s">
+        <v>129</v>
+      </c>
+      <c r="B12" s="13" t="s">
+        <v>181</v>
+      </c>
+      <c r="C12" s="13" t="s">
+        <v>181</v>
+      </c>
+      <c r="D12" s="11" t="s">
+        <v>188</v>
+      </c>
+    </row>
+    <row r="13" spans="1:4" ht="15.75" thickBot="1">
+      <c r="A13" s="8" t="s">
+        <v>130</v>
+      </c>
+      <c r="B13" s="13" t="s">
+        <v>181</v>
+      </c>
+      <c r="C13" s="13" t="s">
+        <v>181</v>
+      </c>
+      <c r="D13" s="11" t="s">
+        <v>189</v>
+      </c>
+    </row>
+    <row r="14" spans="1:4" ht="15.75" thickBot="1">
+      <c r="A14" s="8" t="s">
+        <v>164</v>
+      </c>
+      <c r="B14" s="13" t="s">
+        <v>181</v>
+      </c>
+      <c r="C14" s="13" t="s">
+        <v>181</v>
+      </c>
+      <c r="D14" s="11" t="s">
+        <v>187</v>
+      </c>
+    </row>
+    <row r="15" spans="1:4" ht="15.75" thickBot="1">
+      <c r="A15" s="8" t="s">
+        <v>190</v>
+      </c>
+      <c r="B15" s="13" t="s">
+        <v>181</v>
+      </c>
+      <c r="C15" s="13" t="s">
+        <v>181</v>
+      </c>
+      <c r="D15" s="11" t="s">
+        <v>191</v>
+      </c>
+    </row>
+    <row r="16" spans="1:4" ht="15.75" thickBot="1">
+      <c r="A16" s="8" t="s">
+        <v>169</v>
+      </c>
+      <c r="B16" s="13" t="s">
+        <v>181</v>
+      </c>
+      <c r="C16" s="13" t="s">
+        <v>181</v>
+      </c>
+      <c r="D16" s="11" t="s">
+        <v>191</v>
+      </c>
+    </row>
+    <row r="17" spans="1:4" ht="30.75" thickBot="1">
+      <c r="A17" s="8" t="s">
+        <v>171</v>
+      </c>
+      <c r="B17" s="13" t="s">
+        <v>181</v>
+      </c>
+      <c r="C17" s="14" t="s">
+        <v>186</v>
+      </c>
+      <c r="D17" s="11" t="s">
+        <v>191</v>
+      </c>
+    </row>
+    <row r="18" spans="1:4" ht="15.75" thickBot="1">
+      <c r="A18" s="8" t="s">
+        <v>173</v>
+      </c>
+      <c r="B18" s="13" t="s">
+        <v>181</v>
+      </c>
+      <c r="C18" s="13" t="s">
+        <v>181</v>
+      </c>
+      <c r="D18" s="11" t="s">
+        <v>191</v>
+      </c>
+    </row>
+    <row r="19" spans="1:4" ht="15.75" thickBot="1">
+      <c r="A19" s="8" t="s">
+        <v>192</v>
+      </c>
+      <c r="B19" s="13" t="s">
+        <v>181</v>
+      </c>
+      <c r="C19" s="13" t="s">
+        <v>181</v>
+      </c>
+      <c r="D19" s="11" t="s">
+        <v>187</v>
+      </c>
+    </row>
+    <row r="20" spans="1:4" ht="15.75" thickBot="1">
+      <c r="A20" s="8" t="s">
+        <v>175</v>
+      </c>
+      <c r="B20" s="13" t="s">
+        <v>181</v>
+      </c>
+      <c r="C20" s="13" t="s">
+        <v>181</v>
+      </c>
+      <c r="D20" s="11" t="s">
+        <v>193</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" verticalDpi="0" r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{38B28029-2D30-4424-9CF7-C38ABB644985}">
   <dimension ref="A1:C21"/>
   <sheetFormatPr defaultRowHeight="15"/>
@@ -2195,7 +2705,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{30CA2074-B3C7-4A6C-99A2-8EF34A190107}">
   <dimension ref="A1:B27"/>
   <sheetFormatPr defaultRowHeight="15"/>
@@ -2425,7 +2935,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{29022CD9-CA63-4710-A209-8919E085EC1F}">
   <dimension ref="A1:C17"/>
   <sheetFormatPr defaultRowHeight="15"/>
@@ -2627,7 +3137,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F995789D-50B2-46FE-8AC3-2D0D7F3E1C5E}">
   <dimension ref="A1:B16"/>
   <sheetFormatPr defaultRowHeight="15"/>
@@ -2769,7 +3279,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4177FF4E-0182-40BE-AF37-90E80D22C3E6}">
   <dimension ref="A1:C12"/>
   <sheetFormatPr defaultRowHeight="15"/>

</xml_diff>